<commit_message>
Update demo seed generation logic and documentation
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/server/assets/demo-seed/ar_aging_2026-06-30.xlsx
+++ b/server/assets/demo-seed/ar_aging_2026-06-30.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
-  <si>
-    <t>Brightline Systems Inc. - Accounts Receivable Aging</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
+  <si>
+    <t>Northlight Manufacturing Inc. - Accounts Receivable Aging</t>
   </si>
   <si>
     <t>As of: 2026-06-30</t>
@@ -49,94 +49,100 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Northwind Traders</t>
-  </si>
-  <si>
-    <t>INV-1048</t>
-  </si>
-  <si>
-    <t>2026-06-20</t>
-  </si>
-  <si>
-    <t>2026-07-20</t>
-  </si>
-  <si>
-    <t>Acme Analytics</t>
-  </si>
-  <si>
-    <t>INV-1045</t>
-  </si>
-  <si>
-    <t>2026-06-05</t>
-  </si>
-  <si>
-    <t>2026-07-05</t>
-  </si>
-  <si>
-    <t>Globex Corp</t>
-  </si>
-  <si>
-    <t>INV-1041</t>
-  </si>
-  <si>
-    <t>2026-05-18</t>
-  </si>
-  <si>
-    <t>2026-06-17</t>
-  </si>
-  <si>
-    <t>Initech LLC</t>
-  </si>
-  <si>
-    <t>INV-1038</t>
-  </si>
-  <si>
-    <t>2026-04-28</t>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>BluePeak Distributors LLC</t>
+  </si>
+  <si>
+    <t>NL-2438</t>
+  </si>
+  <si>
+    <t>2026-06-26</t>
+  </si>
+  <si>
+    <t>2026-07-26</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Northgate Assembly LLC</t>
+  </si>
+  <si>
+    <t>NL-2441</t>
+  </si>
+  <si>
+    <t>2026-06-30</t>
+  </si>
+  <si>
+    <t>2026-07-30</t>
+  </si>
+  <si>
+    <t>Helios Retail Group</t>
+  </si>
+  <si>
+    <t>NL-2417</t>
+  </si>
+  <si>
+    <t>2026-05-12</t>
+  </si>
+  <si>
+    <t>2026-06-11</t>
+  </si>
+  <si>
+    <t>partial payment $25,000.00 received 2026-06-15 against $61,500.00</t>
+  </si>
+  <si>
+    <t>Ironwood Fabrication Co</t>
+  </si>
+  <si>
+    <t>NL-2422</t>
   </si>
   <si>
     <t>2026-05-28</t>
   </si>
   <si>
-    <t>Umbrella Health</t>
-  </si>
-  <si>
-    <t>INV-1049</t>
-  </si>
-  <si>
-    <t>2026-06-26</t>
-  </si>
-  <si>
-    <t>2026-07-26</t>
-  </si>
-  <si>
-    <t>Stark Industries</t>
-  </si>
-  <si>
-    <t>INV-1033</t>
-  </si>
-  <si>
-    <t>2026-03-30</t>
-  </si>
-  <si>
-    <t>2026-04-29</t>
-  </si>
-  <si>
-    <t>Wayne Enterprises</t>
-  </si>
-  <si>
-    <t>INV-1027</t>
-  </si>
-  <si>
-    <t>2026-02-12</t>
-  </si>
-  <si>
-    <t>2026-03-14</t>
+    <t>2026-06-27</t>
+  </si>
+  <si>
+    <t>Cascade Equipment Partners</t>
+  </si>
+  <si>
+    <t>NL-2405</t>
+  </si>
+  <si>
+    <t>2026-04-20</t>
+  </si>
+  <si>
+    <t>2026-05-20</t>
+  </si>
+  <si>
+    <t>Sable Ridge Industrial</t>
+  </si>
+  <si>
+    <t>NL-2388</t>
+  </si>
+  <si>
+    <t>2026-03-15</t>
+  </si>
+  <si>
+    <t>2026-04-14</t>
+  </si>
+  <si>
+    <t>Fairmont Tool &amp; Die</t>
+  </si>
+  <si>
+    <t>NL-2361</t>
+  </si>
+  <si>
+    <t>2026-01-30</t>
+  </si>
+  <si>
+    <t>2026-03-01</t>
   </si>
   <si>
     <t>TOTAL</t>
-  </si>
-  <si>
-    <t/>
   </si>
 </sst>
 </file>
@@ -513,7 +519,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -526,7 +532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -557,22 +563,25 @@
       <c r="J4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E5">
-        <v>15200</v>
+        <v>22400</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -587,24 +596,27 @@
         <v>0</v>
       </c>
       <c r="J5">
-        <v>15200</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+        <v>22400</v>
+      </c>
+      <c r="K5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E6">
-        <v>27300</v>
+        <v>18600</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -619,27 +631,30 @@
         <v>0</v>
       </c>
       <c r="J6">
-        <v>27300</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+        <v>18600</v>
+      </c>
+      <c r="K6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
       <c r="F7">
-        <v>12600</v>
+        <v>36500</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -651,30 +666,33 @@
         <v>0</v>
       </c>
       <c r="J7">
-        <v>12600</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+        <v>36500</v>
+      </c>
+      <c r="K7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>14780</v>
       </c>
       <c r="G8">
-        <v>9800</v>
+        <v>0</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -683,30 +701,33 @@
         <v>0</v>
       </c>
       <c r="J8">
-        <v>9800</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+        <v>14780</v>
+      </c>
+      <c r="K8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E9">
-        <v>21150</v>
+        <v>0</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>9340</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -715,21 +736,24 @@
         <v>0</v>
       </c>
       <c r="J9">
-        <v>21150</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+        <v>9340</v>
+      </c>
+      <c r="K9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -741,27 +765,30 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>7450</v>
+        <v>6120</v>
       </c>
       <c r="I10">
         <v>0</v>
       </c>
       <c r="J10">
-        <v>7450</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+        <v>6120</v>
+      </c>
+      <c r="K10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -776,42 +803,48 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>4300</v>
+        <v>3875</v>
       </c>
       <c r="J11">
-        <v>4300</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+        <v>3875</v>
+      </c>
+      <c r="K11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="D12" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="E12">
-        <v>63650</v>
+        <v>41000</v>
       </c>
       <c r="F12">
-        <v>12600</v>
+        <v>51280</v>
       </c>
       <c r="G12">
-        <v>9800</v>
+        <v>9340</v>
       </c>
       <c r="H12">
-        <v>7450</v>
+        <v>6120</v>
       </c>
       <c r="I12">
-        <v>4300</v>
+        <v>3875</v>
       </c>
       <c r="J12">
-        <v>97800</v>
+        <v>111615</v>
+      </c>
+      <c r="K12" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor demo seed generation and update memory fixtures
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/server/assets/demo-seed/ar_aging_2026-06-30.xlsx
+++ b/server/assets/demo-seed/ar_aging_2026-06-30.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
-  <si>
-    <t>Northlight Manufacturing Inc. - Accounts Receivable Aging</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
+  <si>
+    <t>Brightline Systems Inc. - Accounts Receivable Aging</t>
   </si>
   <si>
     <t>As of: 2026-06-30</t>
@@ -49,13 +49,58 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>BluePeak Distributors LLC</t>
-  </si>
-  <si>
-    <t>NL-2438</t>
+    <t>Northwind Traders</t>
+  </si>
+  <si>
+    <t>INV-1048</t>
+  </si>
+  <si>
+    <t>2026-06-20</t>
+  </si>
+  <si>
+    <t>2026-07-20</t>
+  </si>
+  <si>
+    <t>Acme Analytics</t>
+  </si>
+  <si>
+    <t>INV-1045</t>
+  </si>
+  <si>
+    <t>2026-06-05</t>
+  </si>
+  <si>
+    <t>2026-07-05</t>
+  </si>
+  <si>
+    <t>Globex Corp</t>
+  </si>
+  <si>
+    <t>INV-1041</t>
+  </si>
+  <si>
+    <t>2026-05-18</t>
+  </si>
+  <si>
+    <t>2026-06-17</t>
+  </si>
+  <si>
+    <t>Initech LLC</t>
+  </si>
+  <si>
+    <t>INV-1038</t>
+  </si>
+  <si>
+    <t>2026-04-28</t>
+  </si>
+  <si>
+    <t>2026-05-28</t>
+  </si>
+  <si>
+    <t>Umbrella Health</t>
+  </si>
+  <si>
+    <t>INV-1049</t>
   </si>
   <si>
     <t>2026-06-26</t>
@@ -64,85 +109,34 @@
     <t>2026-07-26</t>
   </si>
   <si>
+    <t>Stark Industries</t>
+  </si>
+  <si>
+    <t>INV-1033</t>
+  </si>
+  <si>
+    <t>2026-03-30</t>
+  </si>
+  <si>
+    <t>2026-04-29</t>
+  </si>
+  <si>
+    <t>Wayne Enterprises</t>
+  </si>
+  <si>
+    <t>INV-1027</t>
+  </si>
+  <si>
+    <t>2026-02-12</t>
+  </si>
+  <si>
+    <t>2026-03-14</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>Northgate Assembly LLC</t>
-  </si>
-  <si>
-    <t>NL-2441</t>
-  </si>
-  <si>
-    <t>2026-06-30</t>
-  </si>
-  <si>
-    <t>2026-07-30</t>
-  </si>
-  <si>
-    <t>Helios Retail Group</t>
-  </si>
-  <si>
-    <t>NL-2417</t>
-  </si>
-  <si>
-    <t>2026-05-12</t>
-  </si>
-  <si>
-    <t>2026-06-11</t>
-  </si>
-  <si>
-    <t>partial payment $25,000.00 received 2026-06-15 against $61,500.00</t>
-  </si>
-  <si>
-    <t>Ironwood Fabrication Co</t>
-  </si>
-  <si>
-    <t>NL-2422</t>
-  </si>
-  <si>
-    <t>2026-05-28</t>
-  </si>
-  <si>
-    <t>2026-06-27</t>
-  </si>
-  <si>
-    <t>Cascade Equipment Partners</t>
-  </si>
-  <si>
-    <t>NL-2405</t>
-  </si>
-  <si>
-    <t>2026-04-20</t>
-  </si>
-  <si>
-    <t>2026-05-20</t>
-  </si>
-  <si>
-    <t>Sable Ridge Industrial</t>
-  </si>
-  <si>
-    <t>NL-2388</t>
-  </si>
-  <si>
-    <t>2026-03-15</t>
-  </si>
-  <si>
-    <t>2026-04-14</t>
-  </si>
-  <si>
-    <t>Fairmont Tool &amp; Die</t>
-  </si>
-  <si>
-    <t>NL-2361</t>
-  </si>
-  <si>
-    <t>2026-01-30</t>
-  </si>
-  <si>
-    <t>2026-03-01</t>
-  </si>
-  <si>
-    <t>TOTAL</t>
   </si>
 </sst>
 </file>
@@ -519,7 +513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -532,7 +526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -563,288 +557,261 @@
       <c r="J4" t="s">
         <v>11</v>
       </c>
-      <c r="K4" t="s">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>15</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5">
+        <v>15200</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>15200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>16</v>
       </c>
-      <c r="E5">
-        <v>22400</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
-        <v>22400</v>
-      </c>
-      <c r="K5" t="s">
+      <c r="B6" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="C6" t="s">
         <v>18</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>19</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6">
+        <v>27300</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>27300</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>20</v>
       </c>
-      <c r="D6" t="s">
+      <c r="B7" t="s">
         <v>21</v>
       </c>
-      <c r="E6">
-        <v>18600</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>18600</v>
-      </c>
-      <c r="K6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="C7" t="s">
         <v>22</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>23</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>12600</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>12600</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>24</v>
       </c>
-      <c r="D7" t="s">
+      <c r="B8" t="s">
         <v>25</v>
       </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>36500</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>36500</v>
-      </c>
-      <c r="K7" t="s">
+      <c r="C8" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="D8" t="s">
         <v>27</v>
       </c>
-      <c r="B8" t="s">
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>9800</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>9800</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>28</v>
       </c>
-      <c r="C8" t="s">
+      <c r="B9" t="s">
         <v>29</v>
       </c>
-      <c r="D8" t="s">
+      <c r="C9" t="s">
         <v>30</v>
       </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>14780</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
-        <v>14780</v>
-      </c>
-      <c r="K8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="D9" t="s">
         <v>31</v>
       </c>
-      <c r="B9" t="s">
+      <c r="E9">
+        <v>21150</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>21150</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>32</v>
       </c>
-      <c r="C9" t="s">
+      <c r="B10" t="s">
         <v>33</v>
       </c>
-      <c r="D9" t="s">
+      <c r="C10" t="s">
         <v>34</v>
       </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>9340</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-      <c r="J9">
-        <v>9340</v>
-      </c>
-      <c r="K9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="D10" t="s">
         <v>35</v>
       </c>
-      <c r="B10" t="s">
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>7450</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>7450</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>36</v>
       </c>
-      <c r="C10" t="s">
+      <c r="B11" t="s">
         <v>37</v>
       </c>
-      <c r="D10" t="s">
+      <c r="C11" t="s">
         <v>38</v>
       </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10">
-        <v>6120</v>
-      </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-      <c r="J10">
-        <v>6120</v>
-      </c>
-      <c r="K10" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="D11" t="s">
         <v>39</v>
       </c>
-      <c r="B11" t="s">
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>4300</v>
+      </c>
+      <c r="J11">
+        <v>4300</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>40</v>
       </c>
-      <c r="C11" t="s">
+      <c r="B12" t="s">
         <v>41</v>
       </c>
-      <c r="D11" t="s">
-        <v>42</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11">
-        <v>0</v>
-      </c>
-      <c r="I11">
-        <v>3875</v>
-      </c>
-      <c r="J11">
-        <v>3875</v>
-      </c>
-      <c r="K11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>43</v>
-      </c>
-      <c r="B12" t="s">
-        <v>17</v>
-      </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="E12">
-        <v>41000</v>
+        <v>63650</v>
       </c>
       <c r="F12">
-        <v>51280</v>
+        <v>12600</v>
       </c>
       <c r="G12">
-        <v>9340</v>
+        <v>9800</v>
       </c>
       <c r="H12">
-        <v>6120</v>
+        <v>7450</v>
       </c>
       <c r="I12">
-        <v>3875</v>
+        <v>4300</v>
       </c>
       <c r="J12">
-        <v>111615</v>
-      </c>
-      <c r="K12" t="s">
-        <v>17</v>
+        <v>97800</v>
       </c>
     </row>
   </sheetData>

</xml_diff>